<commit_message>
docs(runbooks): registra a decisão do dono e atende a revisão do PR #53
P1: o runbook mandava corrigir a planilha e reimportar as linhas de telefone
ilegível; o importador de oportunidades não tem dedupe e isso criaria um segundo
card. Agora manda corrigir o card que já entrou e diz, nas duas peças, que cada
arquivo de Oportunidades sobe uma vez só.

P2 de texto: o importador escolhe a primeira etapa ABERTA e só recusa funil sem
etapa aberta (não exige reordenar o quadro); e-mail da linha só é gravado quando
o contato é criado; Audit Log é manager+ e o agent guarda o resumo da tela; a aba
Empresas e pessoas vai como CSV, porque o leitor de .xlsx lê só a primeira aba
(Instruções); tags de oportunidade ficam como escritas, só as de contato viram
minúsculas.

Decisão do dono (2026-10-21): as colunas etapa, produto e origem não serão
implementadas por ora; o desenho futuro está na issue #54.

Refs #52 #54

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/runbooks/modelo-importacao-de-dados.xlsx
+++ b/docs/runbooks/modelo-importacao-de-dados.xlsx
@@ -234,7 +234,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Várias na mesma célula, separadas por ponto e vírgula: quente;retorno. Até 20 por linha. Ficam em letra minúscula.</t>
+          <t xml:space="preserve">Várias na mesma célula, separadas por ponto e vírgula: quente;retorno. Até 20 por linha. Escreva sempre em letra minúscula: na aba Contatos o CRM corrige sozinho; na aba Oportunidades a tag fica como foi escrita, e 'Quente' e 'quente' viram duas tags diferentes.</t>
         </is>
       </c>
     </row>
@@ -346,67 +346,79 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">A oportunidade entra sem contato e a tela avisa a linha. Corrija no card depois ou arrume a planilha.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aba Contexto Green (AINDA NÃO IMPORTÁVEL)</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">A oportunidade entra assim mesmo, sem contato, e a tela avisa a linha. Corrija no card que já entrou (ligue o contato nele). NÃO importe essa linha de novo: viraria um segundo card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não reimporte</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Este importador não reconhece oportunidade repetida: cada linha enviada vira um card novo, mesmo igual a um que já existe. Suba cada arquivo uma vez só e ajuste o que precisar no card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t xml:space="preserve">Aba Contexto Green (AINDA NÃO IMPORTÁVEL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t xml:space="preserve">O que é</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Produto Green e etapa de cada oportunidade. O CRM hoje só grava o produto pela tela, uma oportunidade por vez (dossiê › Produto Green). Esta aba é para você já reunir o dado; o runbook diz como ele entra e qual é o caminho proposto para importar isso.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aba Produtos Green (AINDA NÃO IMPORTÁVEL)</t>
-        </is>
-      </c>
-    </row>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Produto Green e etapa de cada oportunidade. O CRM grava o produto pela tela, uma oportunidade por vez (dossiê › Produto Green), e a etapa se ajusta arrastando o card. Decisão de 21/10/2026: isso segue manual por ora; esta aba é só para você reunir o dado antes de ir para a tela (issue #54 guarda o desenho futuro).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t xml:space="preserve">Aba Produtos Green (AINDA NÃO IMPORTÁVEL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t xml:space="preserve">O que é</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t xml:space="preserve">O catálogo de produtos Green da organização. Cadastre pela tela Configurações › Produtos Green, um por um (são poucos). Regra do código: só letras minúsculas, números e _, começando por letra, 2 a 63 caracteres. O código não pode ser trocado depois.</t>
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aba Empresas e pessoas (OPCIONAL)</t>
-        </is>
-      </c>
-    </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t xml:space="preserve">Aba Empresas e pessoas (OPCIONAL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t xml:space="preserve">O que é</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Só se a instalação tiver o módulo 'Empresas e pessoas (venda para empresas)' ligado em Configurações. Esse importador aceita .xlsx direto (primeira aba) ou CSV, até 2.000 linhas, e só gerente/admin importa.</t>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Só se a instalação tiver o módulo 'Empresas e pessoas (venda para empresas)' ligado em Configurações. Até 2.000 linhas; só gerente/admin importa. Exporte ESTA aba como CSV antes de enviar: esse importador lê só a primeira aba de um .xlsx, e a primeira aba deste arquivo é Instruções.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(runbooks): pausar as automações de negócio criado antes de importar
P1 da terceira rodada do #53: cada oportunidade importada emite `lead.created`
e o motor de automações (`lib/automation/engine.ts`) roda toda regra ativa com
esse gatilho sem distinguir o que veio de planilha; só o gatilho de follow-up
(`lib/followup/gatilho-lead.ts`) ignora a importação. O runbook (seção 2 e
plano da semana) e a aba Instruções passam a mandar pausar essas regras em
Webhooks › Automações antes de subir Oportunidades e religar depois.

Os quatro P2 desta rodada foram para a issue #54, por decisão do dono.

Refs #52 #54

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/runbooks/modelo-importacao-de-dados.xlsx
+++ b/docs/runbooks/modelo-importacao-de-dados.xlsx
@@ -125,298 +125,310 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.</t>
+          <t xml:space="preserve">3a.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deixe as colunas como TEXTO (já vêm assim). Telefone que vira número perde o zero e o +; data que vira data sai em outro formato.</t>
+          <t xml:space="preserve">ANTES de subir Oportunidades, PAUSE as automações disparadas por 'negócio criado' (menu Webhooks › aba Automações; cada regra tem o botão Pausar, e o estado aparece como Ativa ou Pausada). Cada linha importada dispara esse gatilho como se fosse um negócio novo: uma regra que manda WhatsApp ou aciona a IA mandaria 500 mensagens. Religue as regras depois que a importação terminar e você conferir o quadro. (Os follow-ups do funil já ignoram importação; as automações, não.)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.</t>
+          <t xml:space="preserve">4.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Linha com problema é pulada e o motivo aparece na tela, com o número da linha. As outras linhas entram. Corrija só as recusadas e importe de novo o arquivo com elas.</t>
+          <t xml:space="preserve">Deixe as colunas como TEXTO (já vêm assim). Telefone que vira número perde o zero e o +; data que vira data sai em outro formato.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t xml:space="preserve">5.</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linha com problema é pulada e o motivo aparece na tela, com o número da linha. As outras linhas entram. Corrija só as recusadas e importe de novo o arquivo com elas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t xml:space="preserve">6.</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t xml:space="preserve">O passo a passo completo está em docs/runbooks/importar-dados-por-planilha.md.</t>
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Formatos aceitos</t>
-        </is>
-      </c>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Telefone</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Com DDD, com ou sem máscara: 11988887777, (11) 98888-7777 ou +5511988887777. Número só com DDD (10 ou 11 dígitos) ganha +55 sozinho. Número de fora do Brasil precisa vir com + e o código do país.</t>
+          <t xml:space="preserve">Formatos aceitos</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">E-mail</t>
+          <t xml:space="preserve">Telefone</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">formato nome@dominio.com. Letras maiúsculas e minúsculas valem igual para a checagem de repetido.</t>
+          <t xml:space="preserve">Com DDD, com ou sem máscara: 11988887777, (11) 98888-7777 ou +5511988887777. Número só com DDD (10 ou 11 dígitos) ganha +55 sozinho. Número de fora do Brasil precisa vir com + e o código do país.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">CPF</t>
+          <t xml:space="preserve">E-mail</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">11 dígitos, com ou sem pontos e traço: 529.982.247-25 ou 52998224725. O CRM confere o dígito verificador: CPF inventado é recusado. O CPF fica cifrado no banco.</t>
+          <t xml:space="preserve">formato nome@dominio.com. Letras maiúsculas e minúsculas valem igual para a checagem de repetido.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data</t>
+          <t xml:space="preserve">CPF</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">DD/MM/AAAA (31/12/1990) ou AAAA-MM-DD (1990-12-31). Dia que não existe (31/02) é recusado.</t>
+          <t xml:space="preserve">11 dígitos, com ou sem pontos e traço: 529.982.247-25 ou 52998224725. O CRM confere o dígito verificador: CPF inventado é recusado. O CPF fica cifrado no banco.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valor</t>
+          <t xml:space="preserve">Data</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">NA MOEDA CONFIGURADA DA ORGANIZAÇÃO (Configurações › Organização): o CRM não converte, só grava o número com a moeda da organização. Formatos aceitos: 12.500,00 ou 1200 ou R$ 1.200,00 ou 1200.50 ou 1200,50. O último separador com 1 ou 2 dígitos depois é o decimal; com 3 dígitos é milhar (1.200 e 1,200 são mil e duzentos, nunca um e vinte).</t>
+          <t xml:space="preserve">DD/MM/AAAA (31/12/1990) ou AAAA-MM-DD (1990-12-31). Dia que não existe (31/02) é recusado.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tags</t>
+          <t xml:space="preserve">Valor</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Várias na mesma célula, separadas por ponto e vírgula: quente;retorno. Até 20 por linha. Escreva sempre em letra minúscula: na aba Contatos o CRM corrige sozinho; na aba Oportunidades a tag fica como foi escrita, e 'Quente' e 'quente' viram duas tags diferentes.</t>
+          <t xml:space="preserve">NA MOEDA CONFIGURADA DA ORGANIZAÇÃO (Configurações › Organização): o CRM não converte, só grava o número com a moeda da organização. Formatos aceitos: 12.500,00 ou 1200 ou R$ 1.200,00 ou 1200.50 ou 1200,50. O último separador com 1 ou 2 dígitos depois é o decimal; com 3 dígitos é milhar (1.200 e 1,200 são mil e duzentos, nunca um e vinte).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t xml:space="preserve">Tags</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Várias na mesma célula, separadas por ponto e vírgula: quente;retorno. Até 20 por linha. Escreva sempre em letra minúscula: na aba Contatos o CRM corrige sozinho; na aba Oportunidades a tag fica como foi escrita, e 'Quente' e 'quente' viram duas tags diferentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t xml:space="preserve">Origem</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t xml:space="preserve">Texto livre curto, sem acento, que diz por onde a pessoa chegou: indicacao, site, meta_ads, google_ads, whatsapp, evento. Use sempre a mesma grafia para a mesma origem, senão vira duas origens no relatório.</t>
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aba Contatos</t>
-        </is>
-      </c>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obrigatório</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pelo menos telefone OU email em cada linha (de preferência telefone: é por ele que o WhatsApp acha a pessoa).</t>
+          <t xml:space="preserve">Aba Contatos</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Repetidos</t>
+          <t xml:space="preserve">Obrigatório</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Telefone, e-mail ou CPF que já existe no CRM não é criado de novo nem é erro: a linha conta como 'duplicado'.</t>
+          <t xml:space="preserve">Pelo menos telefone OU email em cada linha (de preferência telefone: é por ele que o WhatsApp acha a pessoa).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t xml:space="preserve">Repetidos</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Telefone, e-mail ou CPF que já existe no CRM não é criado de novo nem é erro: a linha conta como 'duplicado'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t xml:space="preserve">Não entra</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t xml:space="preserve">Origem (todo contato importado fica com origem 'import_csv'), empresa, endereço, campos personalizados. Veja o runbook para o que fazer com esses dados.</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aba Oportunidades</t>
-        </is>
-      </c>
-    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obrigatório</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nome (o nome do negócio) OU nome do contato. Escolha o funil na tela na hora de importar.</t>
+          <t xml:space="preserve">Aba Oportunidades</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etapa</t>
+          <t xml:space="preserve">Obrigatório</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toda linha entra na PRIMEIRA etapa aberta do funil escolhido. Não existe coluna de etapa hoje. Para já começar em outra etapa, faça um arquivo por etapa e mova os cards no quadro depois, em seleções de até 50 cards por vez (ou veja a aba 'Contexto Green' e o runbook).</t>
+          <t xml:space="preserve">nome (o nome do negócio) OU nome do contato. Escolha o funil na tela na hora de importar.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contato</t>
+          <t xml:space="preserve">Etapa</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Se o telefone já existe em Contatos, a oportunidade é ligada a ele. Se não existe, o CRM cria o contato com nome do contato, telefone e email.</t>
+          <t xml:space="preserve">Toda linha entra na PRIMEIRA etapa aberta do funil escolhido. Não existe coluna de etapa hoje. Para já começar em outra etapa, faça um arquivo por etapa e mova os cards no quadro depois, em seleções de até 50 cards por vez (ou veja a aba 'Contexto Green' e o runbook).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Telefone errado</t>
+          <t xml:space="preserve">Contato</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">A oportunidade entra assim mesmo, sem contato, e a tela avisa a linha. O card sem contato não tem como ganhar um contato pela tela: apague esse card no quadro e importe de novo SÓ essa linha, com o telefone corrigido. Sem apagar antes, viraria um segundo card.</t>
+          <t xml:space="preserve">Se o telefone já existe em Contatos, a oportunidade é ligada a ele. Se não existe, o CRM cria o contato com nome do contato, telefone e email.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t xml:space="preserve">Telefone errado</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A oportunidade entra assim mesmo, sem contato, e a tela avisa a linha. O card sem contato não tem como ganhar um contato pela tela: apague esse card no quadro e importe de novo SÓ essa linha, com o telefone corrigido. Sem apagar antes, viraria um segundo card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t xml:space="preserve">Não reimporte</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t xml:space="preserve">Este importador não reconhece oportunidade repetida: cada linha enviada vira um card novo, mesmo igual a um que já existe. Suba cada arquivo uma vez só e ajuste o que precisar no card.</t>
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aba Contexto Green (AINDA NÃO IMPORTÁVEL)</t>
-        </is>
-      </c>
-    </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t xml:space="preserve">Aba Contexto Green (AINDA NÃO IMPORTÁVEL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t xml:space="preserve">O que é</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t xml:space="preserve">Produto Green e etapa de cada oportunidade. O CRM grava o produto pela tela, uma oportunidade por vez (dossiê › Produto Green), e a etapa se ajusta arrastando o card. Decisão de 21/10/2026: isso segue manual por ora; esta aba é só para você reunir o dado antes de ir para a tela (issue #54 guarda o desenho futuro).</t>
         </is>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aba Produtos Green (AINDA NÃO IMPORTÁVEL)</t>
-        </is>
-      </c>
-    </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t xml:space="preserve">Aba Produtos Green (AINDA NÃO IMPORTÁVEL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t xml:space="preserve">O que é</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t xml:space="preserve">O catálogo de produtos Green da organização. Cadastre pela tela Configurações › Produtos Green, um por um (são poucos). Regra do código: só letras minúsculas, números e _, começando por letra, 2 a 63 caracteres. O código não pode ser trocado depois.</t>
         </is>
       </c>
     </row>
-    <row r="37"/>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aba Empresas e pessoas (OPCIONAL)</t>
-        </is>
-      </c>
-    </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t xml:space="preserve">Aba Empresas e pessoas (OPCIONAL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t xml:space="preserve">O que é</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t xml:space="preserve">Só se a instalação tiver o módulo 'Empresas e pessoas (venda para empresas)' ligado em Configurações. Até 2.000 linhas; só gerente/admin importa. Exporte ESTA aba como CSV antes de enviar: esse importador lê só a primeira aba de um .xlsx, e a primeira aba deste arquivo é Instruções.</t>
         </is>

</xml_diff>